<commit_message>
cambios graficos spi + inclusion alarma media prioridad + mejoras UX
</commit_message>
<xml_diff>
--- a/Codigos/Windows/Registro Eventos.xlsx
+++ b/Codigos/Windows/Registro Eventos.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -465,7 +465,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CLONIDINA</t>
+          <t>AAA</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -482,7 +482,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>DEXMEDETOMIDINA</t>
+          <t>CLONIDINA</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -499,7 +499,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>DICLOFENAC</t>
+          <t>DEXMEDETOMIDINA</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -516,7 +516,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>DIPIRONA</t>
+          <t>DICLOFENAC</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -533,7 +533,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>FENTANILO</t>
+          <t>DIPIRONA</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -550,7 +550,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>IBUPROFENO</t>
+          <t>FENTANILO</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
@@ -559,7 +559,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>KETAMINA</t>
+          <t>IBUPROFENO</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
@@ -568,7 +568,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>KETOROLAC</t>
+          <t>KETAMINA</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
@@ -577,7 +577,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>LIDOCAÍNA</t>
+          <t>KETOROLAC</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
@@ -586,7 +586,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>MORFINA</t>
+          <t>LIDOCAÍNA</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
@@ -595,7 +595,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>PARACETAMOL</t>
+          <t>MORFINA</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
@@ -604,7 +604,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>REMIFENTANILO</t>
+          <t>PARACETAMOL</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
@@ -613,11 +613,20 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>TRAMADOL</t>
+          <t>REMIFENTANILO</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>TRAMADOL</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
upper() a los ingresos de texto
</commit_message>
<xml_diff>
--- a/Codigos/Windows/Registro Eventos.xlsx
+++ b/Codigos/Windows/Registro Eventos.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -465,7 +465,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>AAA</t>
+          <t>CLONIDINA</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -482,7 +482,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CLONIDINA</t>
+          <t>DEXMEDETOMIDINA</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -499,7 +499,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>DEXMEDETOMIDINA</t>
+          <t>DICLOFENAC</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -516,7 +516,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>DICLOFENAC</t>
+          <t>DIPIRONA</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -533,7 +533,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>DIPIRONA</t>
+          <t>FENTANILO</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -550,7 +550,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>FENTANILO</t>
+          <t>IBUPROFENO</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
@@ -559,7 +559,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>IBUPROFENO</t>
+          <t>KETAMINA</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
@@ -568,7 +568,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>KETAMINA</t>
+          <t>KETOROLAC</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
@@ -577,7 +577,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>KETOROLAC</t>
+          <t>LIDOCAÍNA</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
@@ -586,7 +586,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>LIDOCAÍNA</t>
+          <t>MORFINA</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
@@ -595,7 +595,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>MORFINA</t>
+          <t>PARACETAMOL</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
@@ -604,7 +604,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>PARACETAMOL</t>
+          <t>REMIFENTANILO</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
@@ -613,20 +613,11 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>REMIFENTANILO</t>
+          <t>TRAMADOL</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>TRAMADOL</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr"/>
-      <c r="C16" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>